<commit_message>
Meeting explorations - Created a new folder for SAF
</commit_message>
<xml_diff>
--- a/src/technology/pv-residential-simple/pv-residential-simple.xlsx
+++ b/src/technology/pv-residential-simple/pv-residential-simple.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rhanes\GitHub\tyche\src\technology\pv-residential-simple\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nrel-my.sharepoint.com/personal/tghosh_nrel_gov/Documents/work_NREL/tyche/src/technology/pv-residential-simple/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{896735AC-4845-4B74-874B-0106DE216EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{896735AC-4845-4B74-874B-0106DE216EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98B95582-8AC9-9749-A532-79937C9E2FD5}"/>
   <bookViews>
-    <workbookView xWindow="30990" yWindow="0" windowWidth="17730" windowHeight="16200" firstSheet="1" activeTab="3" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
+    <workbookView xWindow="4880" yWindow="4860" windowWidth="38400" windowHeight="19260" firstSheet="1" activeTab="3" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
   </bookViews>
   <sheets>
     <sheet name="indices" sheetId="1" r:id="rId1"/>
@@ -670,9 +670,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -710,7 +710,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -816,7 +816,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -958,7 +958,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -967,9 +967,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AF3D170-DEC1-4938-B961-67DBF048922E}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -989,7 +989,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1023,7 +1023,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1040,7 +1040,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1057,7 +1057,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1133,9 +1133,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A97C873A-D063-4744-8651-CEF648C63973}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -1161,7 +1161,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1192,17 +1192,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FB20890-62B7-47AF-BA68-650F053D99C5}">
   <dimension ref="A1:G109"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -1225,7 +1225,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1248,7 +1248,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1294,7 +1294,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1337,7 +1337,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1360,7 +1360,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1383,7 +1383,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1475,7 +1475,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1498,7 +1498,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1541,7 +1541,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -1768,7 +1768,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -1791,7 +1791,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -1860,7 +1860,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -1883,7 +1883,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>21</v>
       </c>
@@ -1926,7 +1926,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>21</v>
       </c>
@@ -1949,7 +1949,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>21</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>21</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>21</v>
       </c>
@@ -2018,7 +2018,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>21</v>
       </c>
@@ -2064,7 +2064,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>21</v>
       </c>
@@ -2087,7 +2087,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>21</v>
       </c>
@@ -2110,7 +2110,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>21</v>
       </c>
@@ -2130,7 +2130,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>21</v>
       </c>
@@ -2153,7 +2153,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>21</v>
       </c>
@@ -2176,7 +2176,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>21</v>
       </c>
@@ -2199,7 +2199,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>21</v>
       </c>
@@ -2222,7 +2222,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>21</v>
       </c>
@@ -2245,7 +2245,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>21</v>
       </c>
@@ -2268,7 +2268,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>21</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>21</v>
       </c>
@@ -2314,7 +2314,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>21</v>
       </c>
@@ -2334,7 +2334,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>21</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>21</v>
       </c>
@@ -2380,7 +2380,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>21</v>
       </c>
@@ -2403,7 +2403,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>21</v>
       </c>
@@ -2426,7 +2426,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>21</v>
       </c>
@@ -2449,7 +2449,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>21</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>21</v>
       </c>
@@ -2495,7 +2495,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>21</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>21</v>
       </c>
@@ -2538,7 +2538,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>21</v>
       </c>
@@ -2561,7 +2561,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>21</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>21</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>21</v>
       </c>
@@ -2630,7 +2630,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>21</v>
       </c>
@@ -2653,7 +2653,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>21</v>
       </c>
@@ -2676,7 +2676,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>21</v>
       </c>
@@ -2699,7 +2699,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>21</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>21</v>
       </c>
@@ -2742,7 +2742,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>21</v>
       </c>
@@ -2765,7 +2765,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>21</v>
       </c>
@@ -2788,7 +2788,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>21</v>
       </c>
@@ -2811,7 +2811,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>21</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>21</v>
       </c>
@@ -2857,7 +2857,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>21</v>
       </c>
@@ -2880,7 +2880,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>21</v>
       </c>
@@ -2903,7 +2903,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>21</v>
       </c>
@@ -2926,7 +2926,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>21</v>
       </c>
@@ -2946,7 +2946,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>21</v>
       </c>
@@ -2969,7 +2969,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>21</v>
       </c>
@@ -2992,7 +2992,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>21</v>
       </c>
@@ -3015,7 +3015,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>21</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>21</v>
       </c>
@@ -3061,7 +3061,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>21</v>
       </c>
@@ -3084,7 +3084,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>21</v>
       </c>
@@ -3107,7 +3107,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>21</v>
       </c>
@@ -3130,7 +3130,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>21</v>
       </c>
@@ -3150,7 +3150,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>21</v>
       </c>
@@ -3173,7 +3173,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>21</v>
       </c>
@@ -3196,7 +3196,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>21</v>
       </c>
@@ -3219,7 +3219,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>21</v>
       </c>
@@ -3242,7 +3242,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>21</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>21</v>
       </c>
@@ -3288,7 +3288,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>21</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>21</v>
       </c>
@@ -3334,7 +3334,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>21</v>
       </c>
@@ -3354,7 +3354,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>21</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>21</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>21</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>21</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>21</v>
       </c>
@@ -3469,7 +3469,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>21</v>
       </c>
@@ -3492,7 +3492,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>21</v>
       </c>
@@ -3515,7 +3515,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>21</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>21</v>
       </c>
@@ -3558,7 +3558,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>21</v>
       </c>
@@ -3581,7 +3581,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>21</v>
       </c>
@@ -3604,7 +3604,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>21</v>
       </c>
@@ -3627,7 +3627,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>21</v>
       </c>
@@ -3650,7 +3650,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>21</v>
       </c>
@@ -3681,17 +3681,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9375A35C-8A58-4D70-9436-2E641DE51D25}">
   <dimension ref="A1:G253"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -3714,7 +3714,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -3737,7 +3737,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -3760,7 +3760,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -3783,7 +3783,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -3806,7 +3806,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -3829,7 +3829,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -3852,7 +3852,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -3875,7 +3875,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -3898,7 +3898,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -3921,7 +3921,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -3967,7 +3967,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -3990,7 +3990,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -4013,7 +4013,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -4036,7 +4036,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -4059,7 +4059,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -4082,7 +4082,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -4105,7 +4105,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -4151,7 +4151,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -4174,7 +4174,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -4197,7 +4197,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -4220,7 +4220,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -4243,7 +4243,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -4266,7 +4266,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -4289,7 +4289,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -4312,7 +4312,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -4335,7 +4335,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -4358,7 +4358,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -4381,7 +4381,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -4404,7 +4404,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>21</v>
       </c>
@@ -4427,7 +4427,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>21</v>
       </c>
@@ -4450,7 +4450,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>21</v>
       </c>
@@ -4473,7 +4473,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>21</v>
       </c>
@@ -4496,7 +4496,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>21</v>
       </c>
@@ -4519,7 +4519,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -4542,7 +4542,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>21</v>
       </c>
@@ -4565,7 +4565,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>21</v>
       </c>
@@ -4588,7 +4588,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>21</v>
       </c>
@@ -4611,7 +4611,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>21</v>
       </c>
@@ -4634,7 +4634,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>21</v>
       </c>
@@ -4657,7 +4657,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>21</v>
       </c>
@@ -4680,7 +4680,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>21</v>
       </c>
@@ -4703,7 +4703,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>21</v>
       </c>
@@ -4726,7 +4726,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>21</v>
       </c>
@@ -4749,7 +4749,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>21</v>
       </c>
@@ -4772,7 +4772,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>21</v>
       </c>
@@ -4795,7 +4795,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>21</v>
       </c>
@@ -4818,7 +4818,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>21</v>
       </c>
@@ -4841,7 +4841,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>21</v>
       </c>
@@ -4864,7 +4864,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>21</v>
       </c>
@@ -4887,7 +4887,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>21</v>
       </c>
@@ -4910,7 +4910,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>21</v>
       </c>
@@ -4933,7 +4933,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>21</v>
       </c>
@@ -4956,7 +4956,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>21</v>
       </c>
@@ -4979,7 +4979,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>21</v>
       </c>
@@ -5002,7 +5002,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>21</v>
       </c>
@@ -5025,7 +5025,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>21</v>
       </c>
@@ -5048,7 +5048,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>21</v>
       </c>
@@ -5071,7 +5071,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>21</v>
       </c>
@@ -5094,7 +5094,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>21</v>
       </c>
@@ -5117,7 +5117,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>21</v>
       </c>
@@ -5140,7 +5140,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>21</v>
       </c>
@@ -5163,7 +5163,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>21</v>
       </c>
@@ -5186,7 +5186,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>21</v>
       </c>
@@ -5209,7 +5209,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>21</v>
       </c>
@@ -5232,7 +5232,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>21</v>
       </c>
@@ -5255,7 +5255,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>21</v>
       </c>
@@ -5278,7 +5278,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>21</v>
       </c>
@@ -5301,7 +5301,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>21</v>
       </c>
@@ -5324,7 +5324,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>21</v>
       </c>
@@ -5347,7 +5347,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>21</v>
       </c>
@@ -5370,7 +5370,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>21</v>
       </c>
@@ -5393,7 +5393,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>21</v>
       </c>
@@ -5416,7 +5416,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>21</v>
       </c>
@@ -5439,7 +5439,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>21</v>
       </c>
@@ -5462,7 +5462,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>21</v>
       </c>
@@ -5485,7 +5485,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>21</v>
       </c>
@@ -5508,7 +5508,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>21</v>
       </c>
@@ -5531,7 +5531,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>21</v>
       </c>
@@ -5554,7 +5554,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>21</v>
       </c>
@@ -5577,7 +5577,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>21</v>
       </c>
@@ -5600,7 +5600,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>21</v>
       </c>
@@ -5623,7 +5623,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>21</v>
       </c>
@@ -5646,7 +5646,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>21</v>
       </c>
@@ -5669,7 +5669,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>21</v>
       </c>
@@ -5692,7 +5692,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>21</v>
       </c>
@@ -5715,7 +5715,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>21</v>
       </c>
@@ -5738,7 +5738,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>21</v>
       </c>
@@ -5761,7 +5761,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>21</v>
       </c>
@@ -5784,7 +5784,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>21</v>
       </c>
@@ -5807,7 +5807,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>21</v>
       </c>
@@ -5830,7 +5830,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>21</v>
       </c>
@@ -5853,7 +5853,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>21</v>
       </c>
@@ -5876,7 +5876,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>21</v>
       </c>
@@ -5899,7 +5899,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>21</v>
       </c>
@@ -5922,7 +5922,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>21</v>
       </c>
@@ -5945,7 +5945,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>21</v>
       </c>
@@ -5968,7 +5968,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>21</v>
       </c>
@@ -5991,7 +5991,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>21</v>
       </c>
@@ -6014,7 +6014,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>21</v>
       </c>
@@ -6037,7 +6037,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>21</v>
       </c>
@@ -6060,7 +6060,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>21</v>
       </c>
@@ -6083,7 +6083,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>21</v>
       </c>
@@ -6106,7 +6106,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>21</v>
       </c>
@@ -6129,7 +6129,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>21</v>
       </c>
@@ -6152,7 +6152,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>21</v>
       </c>
@@ -6175,7 +6175,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>21</v>
       </c>
@@ -6198,7 +6198,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>21</v>
       </c>
@@ -6221,7 +6221,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>21</v>
       </c>
@@ -6244,7 +6244,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>21</v>
       </c>
@@ -6267,7 +6267,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>21</v>
       </c>
@@ -6290,7 +6290,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>21</v>
       </c>
@@ -6313,7 +6313,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>21</v>
       </c>
@@ -6336,7 +6336,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>21</v>
       </c>
@@ -6359,7 +6359,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>21</v>
       </c>
@@ -6382,7 +6382,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>21</v>
       </c>
@@ -6405,7 +6405,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>21</v>
       </c>
@@ -6428,7 +6428,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>21</v>
       </c>
@@ -6451,7 +6451,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>21</v>
       </c>
@@ -6474,7 +6474,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>21</v>
       </c>
@@ -6497,7 +6497,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>21</v>
       </c>
@@ -6520,7 +6520,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>21</v>
       </c>
@@ -6543,7 +6543,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>21</v>
       </c>
@@ -6566,7 +6566,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>21</v>
       </c>
@@ -6589,7 +6589,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>21</v>
       </c>
@@ -6612,7 +6612,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>21</v>
       </c>
@@ -6635,7 +6635,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>21</v>
       </c>
@@ -6658,7 +6658,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>21</v>
       </c>
@@ -6681,7 +6681,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>21</v>
       </c>
@@ -6704,7 +6704,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>21</v>
       </c>
@@ -6727,7 +6727,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>21</v>
       </c>
@@ -6750,7 +6750,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>21</v>
       </c>
@@ -6773,7 +6773,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>21</v>
       </c>
@@ -6796,7 +6796,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>21</v>
       </c>
@@ -6819,7 +6819,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>21</v>
       </c>
@@ -6842,7 +6842,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>21</v>
       </c>
@@ -6865,7 +6865,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>21</v>
       </c>
@@ -6888,7 +6888,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>21</v>
       </c>
@@ -6911,7 +6911,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>21</v>
       </c>
@@ -6934,7 +6934,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>21</v>
       </c>
@@ -6957,7 +6957,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>21</v>
       </c>
@@ -6980,7 +6980,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>21</v>
       </c>
@@ -7003,7 +7003,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>21</v>
       </c>
@@ -7026,7 +7026,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>21</v>
       </c>
@@ -7049,7 +7049,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>21</v>
       </c>
@@ -7072,7 +7072,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>21</v>
       </c>
@@ -7095,7 +7095,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>21</v>
       </c>
@@ -7118,7 +7118,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>21</v>
       </c>
@@ -7141,7 +7141,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>21</v>
       </c>
@@ -7164,7 +7164,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>21</v>
       </c>
@@ -7187,7 +7187,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>21</v>
       </c>
@@ -7210,7 +7210,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>21</v>
       </c>
@@ -7233,7 +7233,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>21</v>
       </c>
@@ -7256,7 +7256,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>21</v>
       </c>
@@ -7279,7 +7279,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>21</v>
       </c>
@@ -7302,7 +7302,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>21</v>
       </c>
@@ -7325,7 +7325,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>21</v>
       </c>
@@ -7348,7 +7348,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>21</v>
       </c>
@@ -7371,7 +7371,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>21</v>
       </c>
@@ -7394,7 +7394,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>21</v>
       </c>
@@ -7417,7 +7417,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>21</v>
       </c>
@@ -7440,7 +7440,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>21</v>
       </c>
@@ -7463,7 +7463,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>21</v>
       </c>
@@ -7486,7 +7486,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>21</v>
       </c>
@@ -7509,7 +7509,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>21</v>
       </c>
@@ -7532,7 +7532,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>21</v>
       </c>
@@ -7555,7 +7555,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>21</v>
       </c>
@@ -7578,7 +7578,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>21</v>
       </c>
@@ -7601,7 +7601,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>21</v>
       </c>
@@ -7624,7 +7624,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>21</v>
       </c>
@@ -7647,7 +7647,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>21</v>
       </c>
@@ -7670,7 +7670,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>21</v>
       </c>
@@ -7693,7 +7693,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>21</v>
       </c>
@@ -7716,7 +7716,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>21</v>
       </c>
@@ -7739,7 +7739,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>21</v>
       </c>
@@ -7762,7 +7762,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>21</v>
       </c>
@@ -7785,7 +7785,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>21</v>
       </c>
@@ -7808,7 +7808,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>21</v>
       </c>
@@ -7831,7 +7831,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>21</v>
       </c>
@@ -7854,7 +7854,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>21</v>
       </c>
@@ -7877,7 +7877,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>21</v>
       </c>
@@ -7900,7 +7900,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>21</v>
       </c>
@@ -7923,7 +7923,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>21</v>
       </c>
@@ -7946,7 +7946,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>21</v>
       </c>
@@ -7969,7 +7969,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>21</v>
       </c>
@@ -7992,7 +7992,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>21</v>
       </c>
@@ -8015,7 +8015,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>21</v>
       </c>
@@ -8038,7 +8038,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>21</v>
       </c>
@@ -8061,7 +8061,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>21</v>
       </c>
@@ -8084,7 +8084,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>21</v>
       </c>
@@ -8107,7 +8107,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>21</v>
       </c>
@@ -8130,7 +8130,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>21</v>
       </c>
@@ -8153,7 +8153,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>21</v>
       </c>
@@ -8176,7 +8176,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>21</v>
       </c>
@@ -8199,7 +8199,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>21</v>
       </c>
@@ -8222,7 +8222,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>21</v>
       </c>
@@ -8245,7 +8245,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>21</v>
       </c>
@@ -8268,7 +8268,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>21</v>
       </c>
@@ -8291,7 +8291,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>21</v>
       </c>
@@ -8314,7 +8314,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>21</v>
       </c>
@@ -8337,7 +8337,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>21</v>
       </c>
@@ -8360,7 +8360,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>21</v>
       </c>
@@ -8383,7 +8383,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>21</v>
       </c>
@@ -8406,7 +8406,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>21</v>
       </c>
@@ -8429,7 +8429,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>21</v>
       </c>
@@ -8452,7 +8452,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>21</v>
       </c>
@@ -8475,7 +8475,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>21</v>
       </c>
@@ -8498,7 +8498,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>21</v>
       </c>
@@ -8521,7 +8521,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>21</v>
       </c>
@@ -8544,7 +8544,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>21</v>
       </c>
@@ -8567,7 +8567,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>21</v>
       </c>
@@ -8590,7 +8590,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>21</v>
       </c>
@@ -8613,7 +8613,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>21</v>
       </c>
@@ -8636,7 +8636,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>21</v>
       </c>
@@ -8659,7 +8659,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>21</v>
       </c>
@@ -8682,7 +8682,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>21</v>
       </c>
@@ -8705,7 +8705,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>21</v>
       </c>
@@ -8728,7 +8728,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>21</v>
       </c>
@@ -8751,7 +8751,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>21</v>
       </c>
@@ -8774,7 +8774,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>21</v>
       </c>
@@ -8797,7 +8797,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>21</v>
       </c>
@@ -8820,7 +8820,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>21</v>
       </c>
@@ -8843,7 +8843,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>21</v>
       </c>
@@ -8866,7 +8866,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>21</v>
       </c>
@@ -8889,7 +8889,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>21</v>
       </c>
@@ -8912,7 +8912,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>21</v>
       </c>
@@ -8935,7 +8935,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>21</v>
       </c>
@@ -8958,7 +8958,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>21</v>
       </c>
@@ -8981,7 +8981,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>21</v>
       </c>
@@ -9004,7 +9004,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>21</v>
       </c>
@@ -9027,7 +9027,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>21</v>
       </c>
@@ -9050,7 +9050,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>21</v>
       </c>
@@ -9073,7 +9073,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>21</v>
       </c>
@@ -9096,7 +9096,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>21</v>
       </c>
@@ -9119,7 +9119,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>21</v>
       </c>
@@ -9142,7 +9142,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>21</v>
       </c>
@@ -9165,7 +9165,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>21</v>
       </c>
@@ -9188,7 +9188,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>21</v>
       </c>
@@ -9211,7 +9211,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>21</v>
       </c>
@@ -9234,7 +9234,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>21</v>
       </c>
@@ -9257,7 +9257,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>21</v>
       </c>
@@ -9280,7 +9280,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>21</v>
       </c>
@@ -9303,7 +9303,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>21</v>
       </c>
@@ -9326,7 +9326,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>21</v>
       </c>
@@ -9349,7 +9349,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>21</v>
       </c>
@@ -9372,7 +9372,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>21</v>
       </c>
@@ -9395,7 +9395,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>21</v>
       </c>
@@ -9418,7 +9418,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>21</v>
       </c>
@@ -9441,7 +9441,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>21</v>
       </c>
@@ -9464,7 +9464,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>21</v>
       </c>
@@ -9487,7 +9487,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>21</v>
       </c>
@@ -9518,9 +9518,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08421A62-7A7F-4754-940E-DE21752714F2}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="46.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -9537,7 +9540,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -9551,7 +9554,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -9565,7 +9568,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -9582,7 +9585,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -9599,7 +9602,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -9624,15 +9627,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D89E1871-0EA4-4433-AFC4-28BCC91530B9}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9646,7 +9649,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -9657,7 +9660,7 @@
         <v>1500000</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -9668,7 +9671,7 @@
         <v>3000000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -9679,7 +9682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -9690,7 +9693,7 @@
         <v>4500000</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -9701,7 +9704,7 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -9712,7 +9715,7 @@
         <v>2000000</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -9723,7 +9726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -9734,7 +9737,7 @@
         <v>3000000</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -9745,7 +9748,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -9756,7 +9759,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -9767,7 +9770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -9786,15 +9789,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD318B56-38BD-4E5D-86D7-782D60429334}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>151</v>
       </c>
@@ -9808,7 +9811,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -9819,7 +9822,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -9830,7 +9833,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>45</v>
       </c>
@@ -9841,7 +9844,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>152</v>
       </c>
@@ -9852,7 +9855,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>152</v>
       </c>
@@ -9863,7 +9866,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>152</v>
       </c>
@@ -9874,7 +9877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>153</v>
       </c>
@@ -9885,7 +9888,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>153</v>
       </c>
@@ -9896,7 +9899,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>153</v>
       </c>
@@ -9907,7 +9910,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>154</v>
       </c>
@@ -9918,7 +9921,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>154</v>
       </c>
@@ -9929,7 +9932,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>154</v>
       </c>
@@ -9943,4 +9946,10 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{95965d95-ecc0-4720-b759-1f33c42ed7da}" enabled="1" method="Standard" siteId="{a0f29d7e-28cd-4f54-8442-7885aee7c080}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>